<commit_message>
Final version: updated package, campaign comparisons, 2026 article, archived experiments
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Experiments_and_package/Experimental_data.xlsx
+++ b/Experiments_and_package/Experimental_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02ff00bc61bfec36/DAE Model Analysis/M_smegmatis_DAE_2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/02ff00bc61bfec36/DAE Model Analysis/DAE_System_Model_Calibration_and_Validation/Experiments_and_package/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="11_9595CCCB5F96CA554F11C8179BBD7EA587F59ABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27007387-80FE-4816-BD44-9780F6DD487B}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="11_9595CCCB5F96CA554F11C8179BBD7EA587F59ABE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1EB56985-EF6D-4D34-A46E-A3DD9D0AA30F}"/>
   <bookViews>
-    <workbookView xWindow="15615" yWindow="4515" windowWidth="11985" windowHeight="10275" tabRatio="870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="750" windowWidth="29040" windowHeight="16440" tabRatio="870" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PE_Normal" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="18">
   <si>
     <t>X</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>Ammonia-deficient (repetition)</t>
-  </si>
-  <si>
-    <t>N (original)</t>
   </si>
   <si>
     <t>Time (Hours)</t>
@@ -574,13 +571,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="21" t="s">
         <v>1</v>
@@ -589,7 +586,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>1</v>
@@ -598,7 +595,7 @@
         <v>3</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J1" s="21" t="s">
         <v>1</v>
@@ -607,7 +604,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="21" t="s">
         <v>1</v>
@@ -1076,7 +1073,7 @@
         <v>4.7133895361573911E-7</v>
       </c>
       <c r="O11" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1114,7 +1111,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1498,13 +1495,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -1513,7 +1510,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -1522,7 +1519,7 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>1</v>
@@ -1531,7 +1528,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>1</v>
@@ -1540,7 +1537,7 @@
         <v>5</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1993,7 +1990,7 @@
         <v>3.743978389823804E-7</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2029,13 +2026,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -2044,7 +2041,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -2053,7 +2050,7 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>1</v>
@@ -2062,7 +2059,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>1</v>
@@ -2071,7 +2068,7 @@
         <v>5</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2524,7 +2521,7 @@
         <v>1.2589254117941658E-5</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2547,13 +2544,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -2562,7 +2559,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -2571,7 +2568,7 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>1</v>
@@ -2580,7 +2577,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>1</v>
@@ -2589,7 +2586,7 @@
         <v>5</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3042,7 +3039,7 @@
         <v>3.28599324760064E-7</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -3065,13 +3062,13 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -3080,7 +3077,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>1</v>
@@ -3089,7 +3086,7 @@
         <v>3</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>1</v>
@@ -3098,7 +3095,7 @@
         <v>4</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
         <v>1</v>
@@ -3107,7 +3104,7 @@
         <v>5</v>
       </c>
       <c r="O1" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -3560,7 +3557,7 @@
         <v>3.8904514499428046E-5</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -3573,7 +3570,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="5" width="14.140625" style="7" bestFit="1" customWidth="1"/>
@@ -3584,9 +3581,9 @@
     <col min="12" max="12" width="13.5703125" style="15" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3615,11 +3612,9 @@
       <c r="J1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M1" s="15"/>
+    </row>
+    <row r="2" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -3651,11 +3646,9 @@
         <f t="shared" ref="J2:J11" si="0">10^-H2</f>
         <v>6.5564184941798275E-8</v>
       </c>
-      <c r="L2" s="12">
-        <v>1.0266189000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M2" s="15"/>
+    </row>
+    <row r="3" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>7</v>
       </c>
@@ -3687,11 +3680,9 @@
         <f t="shared" si="0"/>
         <v>7.7031200579721308E-8</v>
       </c>
-      <c r="L3" s="12">
-        <v>0.98144826666666651</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>16</v>
       </c>
@@ -3723,11 +3714,9 @@
         <f t="shared" si="0"/>
         <v>1.4791083881682016E-7</v>
       </c>
-      <c r="L4" s="12">
-        <v>0.95632079999999997</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M4" s="15"/>
+    </row>
+    <row r="5" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>27.5</v>
       </c>
@@ -3759,11 +3748,9 @@
         <f t="shared" si="0"/>
         <v>3.0902954325135797E-7</v>
       </c>
-      <c r="L5" s="12">
-        <v>0.93993176666666667</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M5" s="15"/>
+    </row>
+    <row r="6" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>40</v>
       </c>
@@ -3795,11 +3782,9 @@
         <f t="shared" si="0"/>
         <v>3.0432198871077237E-7</v>
       </c>
-      <c r="L6" s="14">
-        <v>0.96890796666666679</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>51.5</v>
       </c>
@@ -3832,11 +3817,9 @@
         <f t="shared" si="0"/>
         <v>3.1866424217867213E-7</v>
       </c>
-      <c r="L7" s="14">
-        <v>1.0654959333333334</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>64</v>
       </c>
@@ -3868,11 +3851,9 @@
         <f t="shared" si="0"/>
         <v>3.0902954325135797E-7</v>
       </c>
-      <c r="L8" s="12">
-        <v>0.89976849999999997</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M8" s="15"/>
+    </row>
+    <row r="9" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>75.5</v>
       </c>
@@ -3904,11 +3885,9 @@
         <f t="shared" si="0"/>
         <v>4.0426548736234359E-7</v>
       </c>
-      <c r="L9" s="14">
-        <v>0.95347746666666666</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M9" s="15"/>
+    </row>
+    <row r="10" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>88</v>
       </c>
@@ -3940,11 +3919,9 @@
         <f t="shared" si="0"/>
         <v>3.440857338265124E-7</v>
       </c>
-      <c r="L10" s="14">
-        <v>0.92782166666666654</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M10" s="15"/>
+    </row>
+    <row r="11" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>99.5</v>
       </c>
@@ -3977,9 +3954,40 @@
         <v>4.1368204023885066E-7</v>
       </c>
       <c r="K11" s="6"/>
-      <c r="L11" s="12">
-        <v>0.94822186666666664</v>
-      </c>
+      <c r="M11" s="15"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M12" s="15"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M13" s="15"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M14" s="15"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M15" s="15"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M16" s="15"/>
+    </row>
+    <row r="17" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M17" s="15"/>
+    </row>
+    <row r="18" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M18" s="15"/>
+    </row>
+    <row r="19" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M19" s="15"/>
+    </row>
+    <row r="20" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M20" s="15"/>
+    </row>
+    <row r="21" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M21" s="15"/>
+    </row>
+    <row r="22" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M22" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4000,7 +4008,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -4384,7 +4392,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -4766,7 +4774,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>

</xml_diff>